<commit_message>
Marrero 3: fix mislabeled asset descriptions on both Sayres sheets (said Gentry, a template leftover); 36 labels, values unchanged; re-embed in portal, rebuild bundle
</commit_message>
<xml_diff>
--- a/workbooks/3115/Marrero3_CostSeg_3115_Format.xlsx
+++ b/workbooks/3115/Marrero3_CostSeg_3115_Format.xlsx
@@ -644,52 +644,52 @@
     <t xml:space="preserve">Landscaping</t>
   </si>
   <si>
-    <t xml:space="preserve">Asset #23 - Building - Gentry</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Asset #22 - Land Improvements - Gentry</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Asset #24 - Equipment - Gentry</t>
+    <t xml:space="preserve">Asset #23 - Building - Sayres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asset #22 - Land Improvements - Sayres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asset #24 - Equipment - Sayres</t>
   </si>
   <si>
     <t xml:space="preserve">32 Identical Units - Totals:</t>
   </si>
   <si>
-    <t xml:space="preserve">22 - Land Improvements - Gentry</t>
-  </si>
-  <si>
-    <t xml:space="preserve">23 - Building - Gentry</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24 - Equipment - Gentry</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22 - Land Improvements - Gentry - 5yr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22 - Land Improvements - Gentry - 15yr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22 - Land Improvements - Gentry - 27.5yr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">23 - Building - Gentry - 5yr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">23 - Building - Gentry - 15yr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">23 - Building - Gentry - 27.5yr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24 - Equipment - Gentry - 5yr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24 - Equipment - Gentry - 15yr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24 - Equipment - Gentry - 27.5yr</t>
+    <t xml:space="preserve">22 - Land Improvements - Sayres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23 - Building - Sayres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24 - Equipment - Sayres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22 - Land Improvements - Sayres - 5yr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22 - Land Improvements - Sayres - 15yr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22 - Land Improvements - Sayres - 27.5yr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23 - Building - Sayres - 5yr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23 - Building - Sayres - 15yr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23 - Building - Sayres - 27.5yr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24 - Equipment - Sayres - 5yr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24 - Equipment - Sayres - 15yr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24 - Equipment - Sayres - 27.5yr</t>
   </si>
   <si>
     <t xml:space="preserve">Cost Segregation Study - 6800 Sayres Ave</t>

</xml_diff>